<commit_message>
Add Illuminate and Borderless CBS finds; correct two stale roles
Deep roster sweep: Peter Hung (Illuminate, CBS - confirmed),
Patrick O'Kain (Borderless NY partner, CBS MBA - confirmed),
Ariel Muslera (ex-Borderless LATAM lead, CBS MBA w/ Honors),
James Barone (ex-Illuminate MBA intern, CVF '23-24). Corrected:
Charlton Hook appears to have moved to Crossover Markets;
Brett Palatiello's Illuminate link unverified.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WXzZsq4Qrn4tV9mBn34Mo
</commit_message>
<xml_diff>
--- a/CBS_Crypto_Recruiting_Database.xlsx
+++ b/CBS_Crypto_Recruiting_Database.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16353" uniqueCount="6874">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16377" uniqueCount="6891">
   <si>
     <t xml:space="preserve">Fund</t>
   </si>
@@ -18605,19 +18605,22 @@
     <t xml:space="preserve">Charlton Hook</t>
   </si>
   <si>
-    <t xml:space="preserve">Investment Executive — digital assets (led Kiln Series A; Crossover Markets)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBS MBA '21 — CONFIRMED; thesis bullseye + alumni tie in one person</t>
+    <t xml:space="preserve">Crossover Markets (ex-Illuminate Financial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Appears to have LEFT Illuminate for portfolio co. Crossover Markets (crypto ECN, CROSSx) - verify; CFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBS MBA '21 - CONFIRMED; now inside a market-structure operator: arguably a better door for your thesis, not a worse one</t>
   </si>
   <si>
     <t xml:space="preserve">Brett Palatiello</t>
   </si>
   <si>
-    <t xml:space="preserve">Investment Executive, digital asset capital markets (verify current role)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBS MBA '22 — verify; LinkedIn may show a move</t>
+    <t xml:space="preserve">Illuminate link NOT publicly corroborated (prior: Interplay, Eigen Labs, Spring Valley) - verify on LinkedIn before citing the firm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBS - LinkedIn shows CBS as current/most recent affiliation; treat firm as unverified</t>
   </si>
   <si>
     <t xml:space="preserve">Shazeem Kudchiwala</t>
@@ -18804,6 +18807,54 @@
   </si>
   <si>
     <t xml:space="preserve">Near-peer CBS student — CVF intel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peter Hung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senior Associate, NYC (AI infra &amp; apps); 2026 signals suggest a recent move to Seedcamp US - verify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBS graduate - CONFIRMED; the junior Illuminate door (or Seedcamp US door) either way</t>
+  </si>
+  <si>
+    <t xml:space="preserve">James Barone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ServiceNow (ex-Illuminate Financial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director, Strategic Initiatives; was Illuminate MBA Associate intern (Summer '23, B2B payments)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC; CBS/CVF channels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBS MBA + Columbia Venture Fellow '23-24 - the 'how to land the Illuminate MBA internship' coffee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrick O'Kain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner (New York-based); joined from RW3 Ventures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBS MBA (Finance) - CONFIRMED (3 sources); the Borderless door, NYC-based</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ariel Muslera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bluelabel Ventures (ex-Borderless Capital)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founder; was Lead Partner of Borderless's LATAM fund; Kauffman Fellow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LatAm network</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBS MBA with Honors - CONFIRMED; LATAM crypto VC + CBS = your Brazil angle personified</t>
   </si>
   <si>
     <t xml:space="preserve">Limited to publicly prominent, stable figures named in the Aug 2026 research and tracker; roles change fast in this market, so ALWAYS verify on LinkedIn before outreach and log the verified profile in column G. Where a firm has a platform/careers channel, lead with the firm, not the founder. The Talos and Dragonfly caution rows are non-negotiable. Rows 63 onward added Aug 22, 2026 from general knowledge (Jan 2026 horizon) alongside the universe expansion - verify roles before outreach. CBS-alumni rows added Aug 29, 2026 from a 5-agent web sweep: quotes were verified against cited sources via search snippets; ALWAYS re-verify role and school on LinkedIn before outreach.</t>
@@ -65590,135 +65641,135 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>6839</v>
+        <v>6856</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="47" t="s">
-        <v>6840</v>
+        <v>6857</v>
       </c>
       <c r="B3" s="47" t="s">
-        <v>6841</v>
+        <v>6858</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>6842</v>
+        <v>6859</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>6843</v>
+        <v>6860</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>6844</v>
+        <v>6861</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>6845</v>
+        <v>6862</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>6846</v>
+        <v>6863</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>6847</v>
+        <v>6864</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>6848</v>
+        <v>6865</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>6849</v>
+        <v>6866</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>6850</v>
+        <v>6867</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>6851</v>
+        <v>6868</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>6852</v>
+        <v>6869</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>6853</v>
+        <v>6870</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>6854</v>
+        <v>6871</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>6855</v>
+        <v>6872</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>6856</v>
+        <v>6873</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>6857</v>
+        <v>6874</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>6858</v>
+        <v>6875</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>6859</v>
+        <v>6876</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>6860</v>
+        <v>6877</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>6861</v>
+        <v>6878</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>6862</v>
+        <v>6879</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>6863</v>
+        <v>6880</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>6864</v>
+        <v>6881</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>6865</v>
+        <v>6882</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>6866</v>
+        <v>6883</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>6867</v>
+        <v>6884</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>6868</v>
+        <v>6885</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>6869</v>
+        <v>6886</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>6870</v>
+        <v>6887</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>6871</v>
+        <v>6888</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>6872</v>
+        <v>6889</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>6873</v>
+        <v>6890</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -71833,7 +71884,7 @@
     <tabColor rgb="FF3B7D6E"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="20"/>
@@ -71866,8 +71917,8 @@
         <v>5918</v>
       </c>
       <c r="F3" s="34" t="n">
-        <f aca="false">COUNTA($A$6:$A$111)</f>
-        <v>106</v>
+        <f aca="false">COUNTA($A$6:$A$115)</f>
+        <v>110</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -74000,7 +74051,7 @@
       <c r="J89" s="38"/>
       <c r="K89" s="38"/>
     </row>
-    <row r="90" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="36" t="s">
         <v>6169</v>
       </c>
@@ -74050,7 +74101,7 @@
       <c r="J91" s="38"/>
       <c r="K91" s="38"/>
     </row>
-    <row r="92" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="36" t="s">
         <v>6178</v>
       </c>
@@ -74075,7 +74126,7 @@
       <c r="J92" s="38"/>
       <c r="K92" s="38"/>
     </row>
-    <row r="93" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="36" t="s">
         <v>6181</v>
       </c>
@@ -74100,7 +74151,7 @@
       <c r="J93" s="38"/>
       <c r="K93" s="38"/>
     </row>
-    <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="36" t="s">
         <v>6185</v>
       </c>
@@ -74125,15 +74176,15 @@
       <c r="J94" s="38"/>
       <c r="K94" s="38"/>
     </row>
-    <row r="95" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="36" t="s">
         <v>6188</v>
       </c>
       <c r="B95" s="37" t="s">
-        <v>75</v>
+        <v>6189</v>
       </c>
       <c r="C95" s="37" t="s">
-        <v>6189</v>
+        <v>6190</v>
       </c>
       <c r="D95" s="37" t="s">
         <v>976</v>
@@ -74142,7 +74193,7 @@
         <v>76</v>
       </c>
       <c r="F95" s="37" t="s">
-        <v>6190</v>
+        <v>6191</v>
       </c>
       <c r="G95" s="38"/>
       <c r="H95" s="38"/>
@@ -74150,15 +74201,15 @@
       <c r="J95" s="38"/>
       <c r="K95" s="38"/>
     </row>
-    <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="36" t="s">
-        <v>6191</v>
+        <v>6192</v>
       </c>
       <c r="B96" s="37" t="s">
         <v>75</v>
       </c>
       <c r="C96" s="37" t="s">
-        <v>6192</v>
+        <v>6193</v>
       </c>
       <c r="D96" s="37" t="s">
         <v>976</v>
@@ -74167,7 +74218,7 @@
         <v>3</v>
       </c>
       <c r="F96" s="37" t="s">
-        <v>6193</v>
+        <v>6194</v>
       </c>
       <c r="G96" s="38"/>
       <c r="H96" s="38"/>
@@ -74175,15 +74226,15 @@
       <c r="J96" s="38"/>
       <c r="K96" s="38"/>
     </row>
-    <row r="97" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="36" t="s">
-        <v>6194</v>
+        <v>6195</v>
       </c>
       <c r="B97" s="37" t="s">
         <v>86</v>
       </c>
       <c r="C97" s="37" t="s">
-        <v>6195</v>
+        <v>6196</v>
       </c>
       <c r="D97" s="37" t="s">
         <v>976</v>
@@ -74192,7 +74243,7 @@
         <v>6121</v>
       </c>
       <c r="F97" s="37" t="s">
-        <v>6196</v>
+        <v>6197</v>
       </c>
       <c r="G97" s="38"/>
       <c r="H97" s="38"/>
@@ -74200,15 +74251,15 @@
       <c r="J97" s="38"/>
       <c r="K97" s="38"/>
     </row>
-    <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="36" t="s">
-        <v>6197</v>
+        <v>6198</v>
       </c>
       <c r="B98" s="37" t="s">
         <v>574</v>
       </c>
       <c r="C98" s="37" t="s">
-        <v>6198</v>
+        <v>6199</v>
       </c>
       <c r="D98" s="37" t="s">
         <v>976</v>
@@ -74217,7 +74268,7 @@
         <v>3</v>
       </c>
       <c r="F98" s="37" t="s">
-        <v>6199</v>
+        <v>6200</v>
       </c>
       <c r="G98" s="38"/>
       <c r="H98" s="38"/>
@@ -74225,24 +74276,24 @@
       <c r="J98" s="38"/>
       <c r="K98" s="38"/>
     </row>
-    <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="36" t="s">
-        <v>6200</v>
+        <v>6201</v>
       </c>
       <c r="B99" s="37" t="s">
-        <v>6201</v>
+        <v>6202</v>
       </c>
       <c r="C99" s="37" t="s">
-        <v>6202</v>
+        <v>6203</v>
       </c>
       <c r="D99" s="37" t="s">
         <v>976</v>
       </c>
       <c r="E99" s="37" t="s">
-        <v>6203</v>
+        <v>6204</v>
       </c>
       <c r="F99" s="37" t="s">
-        <v>6204</v>
+        <v>6205</v>
       </c>
       <c r="G99" s="38"/>
       <c r="H99" s="38"/>
@@ -74250,15 +74301,15 @@
       <c r="J99" s="38"/>
       <c r="K99" s="38"/>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="36" t="s">
-        <v>6205</v>
+        <v>6206</v>
       </c>
       <c r="B100" s="37" t="s">
-        <v>6206</v>
+        <v>6207</v>
       </c>
       <c r="C100" s="37" t="s">
-        <v>6207</v>
+        <v>6208</v>
       </c>
       <c r="D100" s="37" t="s">
         <v>976</v>
@@ -74267,7 +74318,7 @@
         <v>161</v>
       </c>
       <c r="F100" s="37" t="s">
-        <v>6208</v>
+        <v>6209</v>
       </c>
       <c r="G100" s="38"/>
       <c r="H100" s="38"/>
@@ -74275,24 +74326,24 @@
       <c r="J100" s="38"/>
       <c r="K100" s="38"/>
     </row>
-    <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="36" t="s">
-        <v>6209</v>
+        <v>6210</v>
       </c>
       <c r="B101" s="37" t="s">
         <v>440</v>
       </c>
       <c r="C101" s="37" t="s">
-        <v>6210</v>
+        <v>6211</v>
       </c>
       <c r="D101" s="37" t="s">
         <v>976</v>
       </c>
       <c r="E101" s="37" t="s">
-        <v>6211</v>
+        <v>6212</v>
       </c>
       <c r="F101" s="37" t="s">
-        <v>6212</v>
+        <v>6213</v>
       </c>
       <c r="G101" s="38"/>
       <c r="H101" s="38"/>
@@ -74300,15 +74351,15 @@
       <c r="J101" s="38"/>
       <c r="K101" s="38"/>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="36" t="s">
-        <v>6213</v>
+        <v>6214</v>
       </c>
       <c r="B102" s="37" t="s">
-        <v>6214</v>
+        <v>6215</v>
       </c>
       <c r="C102" s="37" t="s">
-        <v>6215</v>
+        <v>6216</v>
       </c>
       <c r="D102" s="37" t="s">
         <v>976</v>
@@ -74317,7 +74368,7 @@
         <v>161</v>
       </c>
       <c r="F102" s="37" t="s">
-        <v>6216</v>
+        <v>6217</v>
       </c>
       <c r="G102" s="38"/>
       <c r="H102" s="38"/>
@@ -74325,15 +74376,15 @@
       <c r="J102" s="38"/>
       <c r="K102" s="38"/>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="36" t="s">
-        <v>6217</v>
+        <v>6218</v>
       </c>
       <c r="B103" s="37" t="s">
         <v>567</v>
       </c>
       <c r="C103" s="37" t="s">
-        <v>6218</v>
+        <v>6219</v>
       </c>
       <c r="D103" s="37" t="s">
         <v>5933</v>
@@ -74342,7 +74393,7 @@
         <v>3</v>
       </c>
       <c r="F103" s="37" t="s">
-        <v>6219</v>
+        <v>6220</v>
       </c>
       <c r="G103" s="38"/>
       <c r="H103" s="38"/>
@@ -74350,15 +74401,15 @@
       <c r="J103" s="38"/>
       <c r="K103" s="38"/>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="36" t="s">
-        <v>6220</v>
+        <v>6221</v>
       </c>
       <c r="B104" s="37" t="s">
         <v>929</v>
       </c>
       <c r="C104" s="37" t="s">
-        <v>6221</v>
+        <v>6222</v>
       </c>
       <c r="D104" s="37" t="s">
         <v>5933</v>
@@ -74367,7 +74418,7 @@
         <v>3</v>
       </c>
       <c r="F104" s="37" t="s">
-        <v>6222</v>
+        <v>6223</v>
       </c>
       <c r="G104" s="38"/>
       <c r="H104" s="38"/>
@@ -74375,15 +74426,15 @@
       <c r="J104" s="38"/>
       <c r="K104" s="38"/>
     </row>
-    <row r="105" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="36" t="s">
-        <v>6223</v>
+        <v>6224</v>
       </c>
       <c r="B105" s="37" t="s">
-        <v>6224</v>
+        <v>6225</v>
       </c>
       <c r="C105" s="37" t="s">
-        <v>6225</v>
+        <v>6226</v>
       </c>
       <c r="D105" s="37" t="s">
         <v>5933</v>
@@ -74392,7 +74443,7 @@
         <v>3</v>
       </c>
       <c r="F105" s="37" t="s">
-        <v>6226</v>
+        <v>6227</v>
       </c>
       <c r="G105" s="38"/>
       <c r="H105" s="38"/>
@@ -74400,24 +74451,24 @@
       <c r="J105" s="38"/>
       <c r="K105" s="38"/>
     </row>
-    <row r="106" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="36" t="s">
-        <v>6227</v>
+        <v>6228</v>
       </c>
       <c r="B106" s="37" t="s">
-        <v>6228</v>
+        <v>6229</v>
       </c>
       <c r="C106" s="37" t="s">
-        <v>6229</v>
+        <v>6230</v>
       </c>
       <c r="D106" s="37" t="s">
         <v>5933</v>
       </c>
       <c r="E106" s="37" t="s">
-        <v>6230</v>
+        <v>6231</v>
       </c>
       <c r="F106" s="37" t="s">
-        <v>6231</v>
+        <v>6232</v>
       </c>
       <c r="G106" s="38"/>
       <c r="H106" s="38"/>
@@ -74425,24 +74476,24 @@
       <c r="J106" s="38"/>
       <c r="K106" s="38"/>
     </row>
-    <row r="107" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="36" t="s">
-        <v>6232</v>
+        <v>6233</v>
       </c>
       <c r="B107" s="37" t="s">
-        <v>6233</v>
+        <v>6234</v>
       </c>
       <c r="C107" s="37" t="s">
-        <v>6234</v>
+        <v>6235</v>
       </c>
       <c r="D107" s="37" t="s">
         <v>5933</v>
       </c>
       <c r="E107" s="37" t="s">
-        <v>6235</v>
+        <v>6236</v>
       </c>
       <c r="F107" s="37" t="s">
-        <v>6236</v>
+        <v>6237</v>
       </c>
       <c r="G107" s="38"/>
       <c r="H107" s="38"/>
@@ -74450,24 +74501,24 @@
       <c r="J107" s="38"/>
       <c r="K107" s="38"/>
     </row>
-    <row r="108" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="36" t="s">
-        <v>6237</v>
+        <v>6238</v>
       </c>
       <c r="B108" s="37" t="s">
-        <v>6238</v>
+        <v>6239</v>
       </c>
       <c r="C108" s="37" t="s">
-        <v>6239</v>
+        <v>6240</v>
       </c>
       <c r="D108" s="37" t="s">
         <v>5933</v>
       </c>
       <c r="E108" s="37" t="s">
-        <v>6240</v>
+        <v>6241</v>
       </c>
       <c r="F108" s="37" t="s">
-        <v>6241</v>
+        <v>6242</v>
       </c>
       <c r="G108" s="38"/>
       <c r="H108" s="38"/>
@@ -74475,24 +74526,24 @@
       <c r="J108" s="38"/>
       <c r="K108" s="38"/>
     </row>
-    <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="36" t="s">
-        <v>6242</v>
+        <v>6243</v>
       </c>
       <c r="B109" s="37" t="s">
-        <v>6238</v>
+        <v>6239</v>
       </c>
       <c r="C109" s="37" t="s">
-        <v>6243</v>
+        <v>6244</v>
       </c>
       <c r="D109" s="37" t="s">
         <v>5933</v>
       </c>
       <c r="E109" s="37" t="s">
-        <v>6244</v>
+        <v>6245</v>
       </c>
       <c r="F109" s="37" t="s">
-        <v>6245</v>
+        <v>6246</v>
       </c>
       <c r="G109" s="38"/>
       <c r="H109" s="38"/>
@@ -74500,24 +74551,24 @@
       <c r="J109" s="38"/>
       <c r="K109" s="38"/>
     </row>
-    <row r="110" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="36" t="s">
-        <v>6246</v>
+        <v>6247</v>
       </c>
       <c r="B110" s="37" t="s">
-        <v>6247</v>
+        <v>6248</v>
       </c>
       <c r="C110" s="37" t="s">
-        <v>6248</v>
+        <v>6249</v>
       </c>
       <c r="D110" s="37" t="s">
         <v>5933</v>
       </c>
       <c r="E110" s="37" t="s">
-        <v>6249</v>
+        <v>6250</v>
       </c>
       <c r="F110" s="37" t="s">
-        <v>6250</v>
+        <v>6251</v>
       </c>
       <c r="G110" s="38"/>
       <c r="H110" s="38"/>
@@ -74525,24 +74576,24 @@
       <c r="J110" s="38"/>
       <c r="K110" s="38"/>
     </row>
-    <row r="111" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="36" t="s">
-        <v>6251</v>
+        <v>6252</v>
       </c>
       <c r="B111" s="37" t="s">
-        <v>6252</v>
+        <v>6253</v>
       </c>
       <c r="C111" s="37" t="s">
-        <v>6253</v>
+        <v>6254</v>
       </c>
       <c r="D111" s="37" t="s">
         <v>5933</v>
       </c>
       <c r="E111" s="37" t="s">
-        <v>6254</v>
+        <v>6255</v>
       </c>
       <c r="F111" s="37" t="s">
-        <v>6255</v>
+        <v>6256</v>
       </c>
       <c r="G111" s="38"/>
       <c r="H111" s="38"/>
@@ -74550,9 +74601,109 @@
       <c r="J111" s="38"/>
       <c r="K111" s="38"/>
     </row>
+    <row r="112" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="36" t="s">
+        <v>6257</v>
+      </c>
+      <c r="B112" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="C112" s="37" t="s">
+        <v>6258</v>
+      </c>
+      <c r="D112" s="37" t="s">
+        <v>976</v>
+      </c>
+      <c r="E112" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F112" s="37" t="s">
+        <v>6259</v>
+      </c>
+      <c r="G112" s="38"/>
+      <c r="H112" s="38"/>
+      <c r="I112" s="39"/>
+      <c r="J112" s="38"/>
+      <c r="K112" s="38"/>
+    </row>
     <row r="113" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="40" t="s">
-        <v>6256</v>
+      <c r="A113" s="36" t="s">
+        <v>6260</v>
+      </c>
+      <c r="B113" s="37" t="s">
+        <v>6261</v>
+      </c>
+      <c r="C113" s="37" t="s">
+        <v>6262</v>
+      </c>
+      <c r="D113" s="37" t="s">
+        <v>5933</v>
+      </c>
+      <c r="E113" s="37" t="s">
+        <v>6263</v>
+      </c>
+      <c r="F113" s="37" t="s">
+        <v>6264</v>
+      </c>
+      <c r="G113" s="38"/>
+      <c r="H113" s="38"/>
+      <c r="I113" s="39"/>
+      <c r="J113" s="38"/>
+      <c r="K113" s="38"/>
+    </row>
+    <row r="114" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="36" t="s">
+        <v>6265</v>
+      </c>
+      <c r="B114" s="37" t="s">
+        <v>1631</v>
+      </c>
+      <c r="C114" s="37" t="s">
+        <v>6266</v>
+      </c>
+      <c r="D114" s="37" t="s">
+        <v>976</v>
+      </c>
+      <c r="E114" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F114" s="37" t="s">
+        <v>6267</v>
+      </c>
+      <c r="G114" s="38"/>
+      <c r="H114" s="38"/>
+      <c r="I114" s="39"/>
+      <c r="J114" s="38"/>
+      <c r="K114" s="38"/>
+    </row>
+    <row r="115" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="36" t="s">
+        <v>6268</v>
+      </c>
+      <c r="B115" s="37" t="s">
+        <v>6269</v>
+      </c>
+      <c r="C115" s="37" t="s">
+        <v>6270</v>
+      </c>
+      <c r="D115" s="37" t="s">
+        <v>976</v>
+      </c>
+      <c r="E115" s="37" t="s">
+        <v>6271</v>
+      </c>
+      <c r="F115" s="37" t="s">
+        <v>6272</v>
+      </c>
+      <c r="G115" s="38"/>
+      <c r="H115" s="38"/>
+      <c r="I115" s="39"/>
+      <c r="J115" s="38"/>
+      <c r="K115" s="38"/>
+    </row>
+    <row r="117" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="40" t="s">
+        <v>6273</v>
       </c>
     </row>
   </sheetData>
@@ -74587,7 +74738,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>6257</v>
+        <v>6274</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -74599,28 +74750,28 @@
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>6258</v>
+        <v>6275</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>5921</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>6259</v>
+        <v>6276</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>5817</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>6260</v>
+        <v>6277</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>6261</v>
+        <v>6278</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>6262</v>
+        <v>6279</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>6263</v>
+        <v>6280</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74631,22 +74782,22 @@
         <v>5827</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>6264</v>
+        <v>6281</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>6265</v>
+        <v>6282</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>6266</v>
+        <v>6283</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>6267</v>
+        <v>6284</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>6269</v>
+        <v>6286</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74657,22 +74808,22 @@
         <v>5827</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>6270</v>
+        <v>6287</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>6271</v>
+        <v>6288</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>6272</v>
+        <v>6289</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>5843</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>6273</v>
+        <v>6290</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74683,22 +74834,22 @@
         <v>5827</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>6274</v>
+        <v>6291</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>6275</v>
+        <v>6292</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>6276</v>
+        <v>6293</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>5846</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>6277</v>
+        <v>6294</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74709,22 +74860,22 @@
         <v>5827</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>6278</v>
+        <v>6295</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>6279</v>
+        <v>6296</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>6280</v>
+        <v>6297</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>5830</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>6281</v>
+        <v>6298</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74735,22 +74886,22 @@
         <v>5827</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>6274</v>
+        <v>6291</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>6282</v>
+        <v>6299</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>6283</v>
+        <v>6300</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>5830</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>6284</v>
+        <v>6301</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74761,22 +74912,22 @@
         <v>5827</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>6274</v>
+        <v>6291</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>6285</v>
+        <v>6302</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>6283</v>
+        <v>6300</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>5830</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>6286</v>
+        <v>6303</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74787,22 +74938,22 @@
         <v>5827</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>6287</v>
+        <v>6304</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>6288</v>
+        <v>6305</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>6289</v>
+        <v>6306</v>
       </c>
       <c r="F10" s="19" t="s">
         <v>5830</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>6290</v>
+        <v>6307</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74813,22 +74964,22 @@
         <v>5827</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>6274</v>
+        <v>6291</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>6291</v>
+        <v>6308</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>6283</v>
+        <v>6300</v>
       </c>
       <c r="F11" s="19" t="s">
         <v>5830</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>6292</v>
+        <v>6309</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74839,22 +74990,22 @@
         <v>5827</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>6293</v>
+        <v>6310</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>6294</v>
+        <v>6311</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>6295</v>
+        <v>6312</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>5830</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>6268</v>
+        <v>6285</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>6296</v>
+        <v>6313</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74865,22 +75016,22 @@
         <v>5863</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>6297</v>
+        <v>6314</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>6298</v>
+        <v>6315</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>6299</v>
+        <v>6316</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>6300</v>
+        <v>6317</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>6301</v>
+        <v>6318</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>6302</v>
+        <v>6319</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74891,22 +75042,22 @@
         <v>5863</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>6303</v>
+        <v>6320</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>6304</v>
+        <v>6321</v>
       </c>
       <c r="E14" s="25" t="s">
-        <v>6305</v>
+        <v>6322</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>6306</v>
+        <v>6323</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>6307</v>
+        <v>6324</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>6308</v>
+        <v>6325</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74917,22 +75068,22 @@
         <v>5863</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>6309</v>
+        <v>6326</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>6310</v>
+        <v>6327</v>
       </c>
       <c r="E15" s="25" t="s">
         <v>5873</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>6311</v>
+        <v>6328</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>6301</v>
+        <v>6318</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>6312</v>
+        <v>6329</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74943,22 +75094,22 @@
         <v>5863</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>6313</v>
+        <v>6330</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>6314</v>
+        <v>6331</v>
       </c>
       <c r="E16" s="25" t="s">
         <v>5877</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>6315</v>
+        <v>6332</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>6301</v>
+        <v>6318</v>
       </c>
       <c r="H16" s="25" t="s">
-        <v>6316</v>
+        <v>6333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74969,22 +75120,22 @@
         <v>5880</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>6317</v>
+        <v>6334</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>6318</v>
+        <v>6335</v>
       </c>
       <c r="E17" s="28" t="s">
         <v>5882</v>
       </c>
       <c r="F17" s="28" t="s">
-        <v>6319</v>
+        <v>6336</v>
       </c>
       <c r="G17" s="27" t="s">
-        <v>6320</v>
+        <v>6337</v>
       </c>
       <c r="H17" s="28" t="s">
-        <v>6321</v>
+        <v>6338</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -74995,22 +75146,22 @@
         <v>5880</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>6322</v>
+        <v>6339</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>6323</v>
+        <v>6340</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>6324</v>
+        <v>6341</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>6325</v>
+        <v>6342</v>
       </c>
       <c r="G18" s="27" t="s">
-        <v>6326</v>
+        <v>6343</v>
       </c>
       <c r="H18" s="28" t="s">
-        <v>6327</v>
+        <v>6344</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75021,22 +75172,22 @@
         <v>5880</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>6328</v>
+        <v>6345</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>6329</v>
+        <v>6346</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>6330</v>
+        <v>6347</v>
       </c>
       <c r="F19" s="28" t="s">
-        <v>6331</v>
+        <v>6348</v>
       </c>
       <c r="G19" s="27" t="s">
-        <v>6332</v>
+        <v>6349</v>
       </c>
       <c r="H19" s="28" t="s">
-        <v>6333</v>
+        <v>6350</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75047,22 +75198,22 @@
         <v>5880</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>6334</v>
+        <v>6351</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>6335</v>
+        <v>6352</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>6336</v>
+        <v>6353</v>
       </c>
       <c r="F20" s="28" t="s">
-        <v>6337</v>
+        <v>6354</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>6332</v>
+        <v>6349</v>
       </c>
       <c r="H20" s="28" t="s">
-        <v>6338</v>
+        <v>6355</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75076,7 +75227,7 @@
         <v>3</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>6339</v>
+        <v>6356</v>
       </c>
       <c r="E21" s="28" t="s">
         <v>5898</v>
@@ -75085,10 +75236,10 @@
         <v>5899</v>
       </c>
       <c r="G21" s="27" t="s">
-        <v>6301</v>
+        <v>6318</v>
       </c>
       <c r="H21" s="28" t="s">
-        <v>6340</v>
+        <v>6357</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75099,22 +75250,22 @@
         <v>5880</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>6341</v>
+        <v>6358</v>
       </c>
       <c r="D22" s="28" t="s">
-        <v>6342</v>
+        <v>6359</v>
       </c>
       <c r="E22" s="28" t="s">
         <v>5428</v>
       </c>
       <c r="F22" s="28" t="s">
-        <v>6343</v>
+        <v>6360</v>
       </c>
       <c r="G22" s="27" t="s">
-        <v>6301</v>
+        <v>6318</v>
       </c>
       <c r="H22" s="28" t="s">
-        <v>6344</v>
+        <v>6361</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75122,25 +75273,25 @@
         <v>5153</v>
       </c>
       <c r="B23" s="42" t="s">
-        <v>6345</v>
+        <v>6362</v>
       </c>
       <c r="C23" s="43" t="s">
-        <v>6346</v>
+        <v>6363</v>
       </c>
       <c r="D23" s="43" t="s">
-        <v>6347</v>
+        <v>6364</v>
       </c>
       <c r="E23" s="43" t="s">
-        <v>6348</v>
+        <v>6365</v>
       </c>
       <c r="F23" s="43" t="s">
-        <v>6349</v>
+        <v>6366</v>
       </c>
       <c r="G23" s="42" t="s">
-        <v>6350</v>
+        <v>6367</v>
       </c>
       <c r="H23" s="43" t="s">
-        <v>6351</v>
+        <v>6368</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75148,25 +75299,25 @@
         <v>2149</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>6345</v>
+        <v>6362</v>
       </c>
       <c r="C24" s="43" t="s">
-        <v>6352</v>
+        <v>6369</v>
       </c>
       <c r="D24" s="43" t="s">
-        <v>6353</v>
+        <v>6370</v>
       </c>
       <c r="E24" s="43" t="s">
-        <v>6354</v>
+        <v>6371</v>
       </c>
       <c r="F24" s="43" t="s">
-        <v>6355</v>
+        <v>6372</v>
       </c>
       <c r="G24" s="42" t="s">
-        <v>6356</v>
+        <v>6373</v>
       </c>
       <c r="H24" s="43" t="s">
-        <v>6357</v>
+        <v>6374</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75174,25 +75325,25 @@
         <v>5326</v>
       </c>
       <c r="B25" s="42" t="s">
-        <v>6345</v>
+        <v>6362</v>
       </c>
       <c r="C25" s="43" t="s">
-        <v>6358</v>
+        <v>6375</v>
       </c>
       <c r="D25" s="43" t="s">
-        <v>6359</v>
+        <v>6376</v>
       </c>
       <c r="E25" s="43" t="s">
-        <v>6360</v>
+        <v>6377</v>
       </c>
       <c r="F25" s="43" t="s">
-        <v>6361</v>
+        <v>6378</v>
       </c>
       <c r="G25" s="42" t="s">
-        <v>6332</v>
+        <v>6349</v>
       </c>
       <c r="H25" s="43" t="s">
-        <v>6362</v>
+        <v>6379</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75200,25 +75351,25 @@
         <v>5175</v>
       </c>
       <c r="B26" s="42" t="s">
-        <v>6345</v>
+        <v>6362</v>
       </c>
       <c r="C26" s="43" t="s">
-        <v>6363</v>
+        <v>6380</v>
       </c>
       <c r="D26" s="43" t="s">
-        <v>6364</v>
+        <v>6381</v>
       </c>
       <c r="E26" s="43" t="s">
-        <v>6365</v>
+        <v>6382</v>
       </c>
       <c r="F26" s="43" t="s">
-        <v>6366</v>
+        <v>6383</v>
       </c>
       <c r="G26" s="42" t="s">
-        <v>6301</v>
+        <v>6318</v>
       </c>
       <c r="H26" s="43" t="s">
-        <v>6367</v>
+        <v>6384</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75226,25 +75377,25 @@
         <v>5160</v>
       </c>
       <c r="B27" s="42" t="s">
-        <v>6345</v>
+        <v>6362</v>
       </c>
       <c r="C27" s="43" t="s">
-        <v>6368</v>
+        <v>6385</v>
       </c>
       <c r="D27" s="43" t="s">
-        <v>6369</v>
+        <v>6386</v>
       </c>
       <c r="E27" s="43" t="s">
-        <v>6370</v>
+        <v>6387</v>
       </c>
       <c r="F27" s="43" t="s">
-        <v>6371</v>
+        <v>6388</v>
       </c>
       <c r="G27" s="42" t="s">
-        <v>6372</v>
+        <v>6389</v>
       </c>
       <c r="H27" s="43" t="s">
-        <v>6373</v>
+        <v>6390</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75252,25 +75403,25 @@
         <v>5181</v>
       </c>
       <c r="B28" s="42" t="s">
-        <v>6345</v>
+        <v>6362</v>
       </c>
       <c r="C28" s="43" t="s">
-        <v>6374</v>
+        <v>6391</v>
       </c>
       <c r="D28" s="43" t="s">
-        <v>6375</v>
+        <v>6392</v>
       </c>
       <c r="E28" s="43" t="s">
         <v>5184</v>
       </c>
       <c r="F28" s="43" t="s">
-        <v>6376</v>
+        <v>6393</v>
       </c>
       <c r="G28" s="42" t="s">
-        <v>6377</v>
+        <v>6394</v>
       </c>
       <c r="H28" s="43" t="s">
-        <v>6378</v>
+        <v>6395</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75278,25 +75429,25 @@
         <v>67</v>
       </c>
       <c r="B29" s="45" t="s">
-        <v>6379</v>
+        <v>6396</v>
       </c>
       <c r="C29" s="46" t="s">
-        <v>6380</v>
+        <v>6397</v>
       </c>
       <c r="D29" s="46" t="s">
-        <v>6381</v>
+        <v>6398</v>
       </c>
       <c r="E29" s="46" t="s">
-        <v>6382</v>
+        <v>6399</v>
       </c>
       <c r="F29" s="46" t="s">
-        <v>6383</v>
+        <v>6400</v>
       </c>
       <c r="G29" s="45" t="s">
-        <v>6384</v>
+        <v>6401</v>
       </c>
       <c r="H29" s="46" t="s">
-        <v>6385</v>
+        <v>6402</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75304,25 +75455,25 @@
         <v>236</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>6379</v>
+        <v>6396</v>
       </c>
       <c r="C30" s="46" t="s">
-        <v>6386</v>
+        <v>6403</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>6387</v>
+        <v>6404</v>
       </c>
       <c r="E30" s="46" t="s">
-        <v>6388</v>
+        <v>6405</v>
       </c>
       <c r="F30" s="46" t="s">
-        <v>6389</v>
+        <v>6406</v>
       </c>
       <c r="G30" s="45" t="s">
-        <v>6301</v>
+        <v>6318</v>
       </c>
       <c r="H30" s="46" t="s">
-        <v>6390</v>
+        <v>6407</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75330,25 +75481,25 @@
         <v>184</v>
       </c>
       <c r="B31" s="45" t="s">
-        <v>6379</v>
+        <v>6396</v>
       </c>
       <c r="C31" s="46" t="s">
-        <v>6391</v>
+        <v>6408</v>
       </c>
       <c r="D31" s="46" t="s">
-        <v>6392</v>
+        <v>6409</v>
       </c>
       <c r="E31" s="46" t="s">
-        <v>6393</v>
+        <v>6410</v>
       </c>
       <c r="F31" s="46" t="s">
-        <v>6394</v>
+        <v>6411</v>
       </c>
       <c r="G31" s="45" t="s">
-        <v>6395</v>
+        <v>6412</v>
       </c>
       <c r="H31" s="46" t="s">
-        <v>6396</v>
+        <v>6413</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75356,25 +75507,25 @@
         <v>32</v>
       </c>
       <c r="B32" s="45" t="s">
-        <v>6379</v>
+        <v>6396</v>
       </c>
       <c r="C32" s="46" t="s">
-        <v>6397</v>
+        <v>6414</v>
       </c>
       <c r="D32" s="46" t="s">
-        <v>6398</v>
+        <v>6415</v>
       </c>
       <c r="E32" s="46" t="s">
-        <v>6399</v>
+        <v>6416</v>
       </c>
       <c r="F32" s="46" t="s">
-        <v>6400</v>
+        <v>6417</v>
       </c>
       <c r="G32" s="45" t="s">
-        <v>6401</v>
+        <v>6418</v>
       </c>
       <c r="H32" s="46" t="s">
-        <v>6402</v>
+        <v>6419</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75382,25 +75533,25 @@
         <v>42</v>
       </c>
       <c r="B33" s="45" t="s">
-        <v>6379</v>
+        <v>6396</v>
       </c>
       <c r="C33" s="46" t="s">
-        <v>6403</v>
+        <v>6420</v>
       </c>
       <c r="D33" s="46" t="s">
-        <v>6404</v>
+        <v>6421</v>
       </c>
       <c r="E33" s="46" t="s">
-        <v>6405</v>
+        <v>6422</v>
       </c>
       <c r="F33" s="46" t="s">
-        <v>6406</v>
+        <v>6423</v>
       </c>
       <c r="G33" s="45" t="s">
-        <v>6407</v>
+        <v>6424</v>
       </c>
       <c r="H33" s="46" t="s">
-        <v>6408</v>
+        <v>6425</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75408,30 +75559,30 @@
         <v>107</v>
       </c>
       <c r="B34" s="45" t="s">
-        <v>6379</v>
+        <v>6396</v>
       </c>
       <c r="C34" s="46" t="s">
-        <v>6409</v>
+        <v>6426</v>
       </c>
       <c r="D34" s="46" t="s">
-        <v>6410</v>
+        <v>6427</v>
       </c>
       <c r="E34" s="46" t="s">
-        <v>6411</v>
+        <v>6428</v>
       </c>
       <c r="F34" s="46" t="s">
-        <v>6412</v>
+        <v>6429</v>
       </c>
       <c r="G34" s="45" t="s">
-        <v>6407</v>
+        <v>6424</v>
       </c>
       <c r="H34" s="46" t="s">
-        <v>6413</v>
+        <v>6430</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="29" t="s">
-        <v>6414</v>
+        <v>6431</v>
       </c>
       <c r="B36" s="29"/>
       <c r="C36" s="29"/>
@@ -75477,265 +75628,265 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
-        <v>6415</v>
+        <v>6432</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
-        <v>6416</v>
+        <v>6433</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>6417</v>
+        <v>6434</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="35" t="s">
-        <v>6418</v>
+        <v>6435</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>6419</v>
+        <v>6436</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>6420</v>
+        <v>6437</v>
       </c>
       <c r="D5" s="35" t="s">
-        <v>6421</v>
+        <v>6438</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>6422</v>
+        <v>6439</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>6423</v>
+        <v>6440</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="s">
-        <v>6424</v>
+        <v>6441</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>6425</v>
+        <v>6442</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>6426</v>
+        <v>6443</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>6427</v>
+        <v>6444</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>6428</v>
+        <v>6445</v>
       </c>
       <c r="F6" s="38"/>
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="36" t="s">
-        <v>6429</v>
+        <v>6446</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>6430</v>
+        <v>6447</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>6431</v>
+        <v>6448</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>6432</v>
+        <v>6449</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>6433</v>
+        <v>6450</v>
       </c>
       <c r="F7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="36" t="s">
-        <v>6434</v>
+        <v>6451</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>6435</v>
+        <v>6452</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>6436</v>
+        <v>6453</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>6437</v>
+        <v>6454</v>
       </c>
       <c r="E8" s="37"/>
       <c r="F8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="36" t="s">
-        <v>6438</v>
+        <v>6455</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>6439</v>
+        <v>6456</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>6440</v>
+        <v>6457</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>6441</v>
+        <v>6458</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>6442</v>
+        <v>6459</v>
       </c>
       <c r="F9" s="38"/>
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="36" t="s">
-        <v>6443</v>
+        <v>6460</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>6444</v>
+        <v>6461</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>6445</v>
+        <v>6462</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>6446</v>
+        <v>6463</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>6447</v>
+        <v>6464</v>
       </c>
       <c r="F10" s="38"/>
     </row>
     <row r="11" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="36" t="s">
-        <v>6448</v>
+        <v>6465</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>6449</v>
+        <v>6466</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>6450</v>
+        <v>6467</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>6451</v>
+        <v>6468</v>
       </c>
       <c r="E11" s="37"/>
       <c r="F11" s="38"/>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>6452</v>
+        <v>6469</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>6453</v>
+        <v>6470</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>6454</v>
+        <v>6471</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>6455</v>
+        <v>6472</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>6456</v>
+        <v>6473</v>
       </c>
       <c r="F12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="36" t="s">
-        <v>6457</v>
+        <v>6474</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>6458</v>
+        <v>6475</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>6459</v>
+        <v>6476</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>6460</v>
+        <v>6477</v>
       </c>
       <c r="E13" s="37"/>
       <c r="F13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="s">
-        <v>6461</v>
+        <v>6478</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>6462</v>
+        <v>6479</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>6463</v>
+        <v>6480</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>6464</v>
+        <v>6481</v>
       </c>
       <c r="E14" s="37"/>
       <c r="F14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="s">
-        <v>6465</v>
+        <v>6482</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>6466</v>
+        <v>6483</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>6467</v>
+        <v>6484</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>6468</v>
+        <v>6485</v>
       </c>
       <c r="E15" s="37"/>
       <c r="F15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="s">
-        <v>6469</v>
+        <v>6486</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>6470</v>
+        <v>6487</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>6471</v>
+        <v>6488</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>6472</v>
+        <v>6489</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>6473</v>
+        <v>6490</v>
       </c>
       <c r="F16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="36" t="s">
-        <v>6474</v>
+        <v>6491</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>6475</v>
+        <v>6492</v>
       </c>
       <c r="C17" s="37" t="s">
-        <v>6476</v>
+        <v>6493</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>6477</v>
+        <v>6494</v>
       </c>
       <c r="E17" s="37"/>
       <c r="F17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="36" t="s">
-        <v>6478</v>
+        <v>6495</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>6479</v>
+        <v>6496</v>
       </c>
       <c r="C18" s="37" t="s">
-        <v>6480</v>
+        <v>6497</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>6481</v>
+        <v>6498</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>6482</v>
+        <v>6499</v>
       </c>
       <c r="F18" s="38"/>
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="40" t="s">
-        <v>6483</v>
+        <v>6500</v>
       </c>
     </row>
   </sheetData>
@@ -75768,7 +75919,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>6484</v>
+        <v>6501</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -75782,22 +75933,22 @@
         <v>5816</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>6485</v>
+        <v>6502</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>6486</v>
+        <v>6503</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>6487</v>
+        <v>6504</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>6488</v>
+        <v>6505</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>6489</v>
+        <v>6506</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>6490</v>
+        <v>6507</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75814,13 +75965,13 @@
         <v>0</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>6491</v>
+        <v>6508</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>6492</v>
+        <v>6509</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>6493</v>
+        <v>6510</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75837,13 +75988,13 @@
         <v>1</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>6494</v>
+        <v>6511</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>6495</v>
+        <v>6512</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>6496</v>
+        <v>6513</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75860,13 +76011,13 @@
         <v>3</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>6494</v>
+        <v>6511</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>6497</v>
+        <v>6514</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>6498</v>
+        <v>6515</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75883,13 +76034,13 @@
         <v>1</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>6491</v>
+        <v>6508</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>6499</v>
+        <v>6516</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>6500</v>
+        <v>6517</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75906,13 +76057,13 @@
         <v>2</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>6501</v>
+        <v>6518</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>6502</v>
+        <v>6519</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>6503</v>
+        <v>6520</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75929,13 +76080,13 @@
         <v>0</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>6504</v>
+        <v>6521</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>6505</v>
+        <v>6522</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>6506</v>
+        <v>6523</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75952,18 +76103,18 @@
         <v>2</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>6501</v>
+        <v>6518</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>6507</v>
+        <v>6524</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>6508</v>
+        <v>6525</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>6509</v>
+        <v>6526</v>
       </c>
       <c r="B11" s="18" t="n">
         <v>2</v>
@@ -75975,13 +76126,13 @@
         <v>0</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>6510</v>
+        <v>6527</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>6511</v>
+        <v>6528</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>6512</v>
+        <v>6529</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -75998,13 +76149,13 @@
         <v>0</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>6510</v>
+        <v>6527</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>6513</v>
+        <v>6530</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>6514</v>
+        <v>6531</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76021,13 +76172,13 @@
         <v>2</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>6510</v>
+        <v>6527</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>6515</v>
+        <v>6532</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>6516</v>
+        <v>6533</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76044,13 +76195,13 @@
         <v>0</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>6517</v>
+        <v>6534</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>6518</v>
+        <v>6535</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>6519</v>
+        <v>6536</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76067,13 +76218,13 @@
         <v>0</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>6521</v>
+        <v>6538</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>6522</v>
+        <v>6539</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76090,13 +76241,13 @@
         <v>0</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>6523</v>
+        <v>6540</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>6524</v>
+        <v>6541</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76113,13 +76264,13 @@
         <v>1</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>6525</v>
+        <v>6542</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>6526</v>
+        <v>6543</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76136,13 +76287,13 @@
         <v>1</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>6527</v>
+        <v>6544</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>6528</v>
+        <v>6545</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76159,18 +76310,18 @@
         <v>0</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>6529</v>
+        <v>6546</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>6530</v>
+        <v>6547</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>6531</v>
+        <v>6548</v>
       </c>
       <c r="B20" s="18" t="n">
         <v>1</v>
@@ -76182,13 +76333,13 @@
         <v>0</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>6532</v>
+        <v>6549</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>6533</v>
+        <v>6550</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76205,13 +76356,13 @@
         <v>0</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>6534</v>
+        <v>6551</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>6535</v>
+        <v>6552</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76228,18 +76379,18 @@
         <v>0</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>6536</v>
+        <v>6553</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>6537</v>
+        <v>6554</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>6538</v>
+        <v>6555</v>
       </c>
       <c r="B23" s="18" t="n">
         <v>0</v>
@@ -76251,18 +76402,18 @@
         <v>0</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>6539</v>
+        <v>6556</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>6540</v>
+        <v>6557</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>6541</v>
+        <v>6558</v>
       </c>
       <c r="B24" s="18" t="n">
         <v>1</v>
@@ -76274,13 +76425,13 @@
         <v>0</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>6542</v>
+        <v>6559</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>6543</v>
+        <v>6560</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76294,7 +76445,7 @@
     </row>
     <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>6544</v>
+        <v>6561</v>
       </c>
       <c r="B26" s="18"/>
       <c r="C26" s="18"/>
@@ -76305,7 +76456,7 @@
     </row>
     <row r="27" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>6545</v>
+        <v>6562</v>
       </c>
       <c r="B27" s="18" t="n">
         <v>2</v>
@@ -76317,13 +76468,13 @@
         <v>0</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>6494</v>
+        <v>6511</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>6546</v>
+        <v>6563</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>6547</v>
+        <v>6564</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -76340,18 +76491,18 @@
         <v>0</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>6491</v>
+        <v>6508</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>6548</v>
+        <v>6565</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>6549</v>
+        <v>6566</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>6550</v>
+        <v>6567</v>
       </c>
       <c r="B29" s="18" t="n">
         <v>1</v>
@@ -76363,18 +76514,18 @@
         <v>0</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>6510</v>
+        <v>6527</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>6551</v>
+        <v>6568</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>6552</v>
+        <v>6569</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
-        <v>6553</v>
+        <v>6570</v>
       </c>
       <c r="B30" s="18" t="n">
         <v>0</v>
@@ -76386,18 +76537,18 @@
         <v>1</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>6520</v>
+        <v>6537</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>6554</v>
+        <v>6571</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>6555</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="29" t="s">
-        <v>6556</v>
+        <v>6573</v>
       </c>
       <c r="B32" s="29"/>
       <c r="C32" s="29"/>
@@ -76442,7 +76593,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>6557</v>
+        <v>6574</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -76454,33 +76605,33 @@
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>6558</v>
+        <v>6575</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>5094</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>6559</v>
+        <v>6576</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>6560</v>
+        <v>6577</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>6561</v>
+        <v>6578</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>6562</v>
+        <v>6579</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>6563</v>
+        <v>6580</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>6564</v>
+        <v>6581</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>6565</v>
+        <v>6582</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>1340</v>
@@ -76489,24 +76640,24 @@
         <v>5181</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>6566</v>
+        <v>6583</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>6569</v>
+        <v>6586</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>6570</v>
+        <v>6587</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>1340</v>
@@ -76515,24 +76666,24 @@
         <v>5181</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>6571</v>
+        <v>6588</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>6572</v>
+        <v>6589</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>6573</v>
+        <v>6590</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>1340</v>
@@ -76541,24 +76692,24 @@
         <v>5317</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>6574</v>
+        <v>6591</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>6575</v>
+        <v>6592</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>6576</v>
+        <v>6593</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>6577</v>
+        <v>6594</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>6578</v>
+        <v>6595</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>6573</v>
+        <v>6590</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>1340</v>
@@ -76567,24 +76718,24 @@
         <v>5600</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>6579</v>
+        <v>6596</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>6580</v>
+        <v>6597</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>6581</v>
+        <v>6598</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>6582</v>
+        <v>6599</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>6583</v>
+        <v>6600</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>1340</v>
@@ -76593,36 +76744,36 @@
         <v>5712</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>6584</v>
+        <v>6601</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>6585</v>
+        <v>6602</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>6586</v>
+        <v>6603</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>6587</v>
+        <v>6604</v>
       </c>
       <c r="H8" s="19" t="s">
-        <v>6588</v>
+        <v>6605</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>6589</v>
+        <v>6606</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>6590</v>
+        <v>6607</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>6591</v>
+        <v>6608</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>6592</v>
+        <v>6609</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>5896</v>
@@ -76634,7 +76785,7 @@
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>6589</v>
+        <v>6606</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>1340</v>
@@ -76643,24 +76794,24 @@
         <v>5107</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>6593</v>
+        <v>6610</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>6594</v>
+        <v>6611</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>6595</v>
+        <v>6612</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>1340</v>
@@ -76669,36 +76820,36 @@
         <v>5326</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>6596</v>
+        <v>6613</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>6597</v>
+        <v>6614</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>6598</v>
+        <v>6615</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>6599</v>
+        <v>6616</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>6600</v>
+        <v>6617</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>6601</v>
+        <v>6618</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>6602</v>
+        <v>6619</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>5859</v>
@@ -76707,12 +76858,12 @@
         <v>5837</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>6603</v>
+        <v>6620</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>6599</v>
+        <v>6616</v>
       </c>
       <c r="B13" s="18" t="s">
         <v>1340</v>
@@ -76721,24 +76872,24 @@
         <v>5332</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>6604</v>
+        <v>6621</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>6605</v>
+        <v>6622</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>6606</v>
+        <v>6623</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>6607</v>
+        <v>6624</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>6608</v>
+        <v>6625</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>1340</v>
@@ -76747,24 +76898,24 @@
         <v>5175</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>6609</v>
+        <v>6626</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>6610</v>
+        <v>6627</v>
       </c>
       <c r="F14" s="19" t="s">
         <v>5867</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H14" s="19" t="s">
-        <v>6611</v>
+        <v>6628</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>6612</v>
+        <v>6629</v>
       </c>
       <c r="B15" s="18" t="s">
         <v>1340</v>
@@ -76773,24 +76924,24 @@
         <v>2149</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>6613</v>
+        <v>6630</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>6614</v>
+        <v>6631</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>5867</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>6615</v>
+        <v>6632</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>6612</v>
+        <v>6629</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>1340</v>
@@ -76799,50 +76950,50 @@
         <v>5317</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>6616</v>
+        <v>6633</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>6617</v>
+        <v>6634</v>
       </c>
       <c r="F16" s="19" t="s">
         <v>5867</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>6550</v>
+        <v>6567</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>6618</v>
+        <v>6635</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>6619</v>
+        <v>6636</v>
       </c>
       <c r="B17" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>6620</v>
+        <v>6637</v>
       </c>
       <c r="D17" s="19" t="s">
         <v>5797</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>6621</v>
+        <v>6638</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>6622</v>
+        <v>6639</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>6545</v>
+        <v>6562</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>6623</v>
+        <v>6640</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>6619</v>
+        <v>6636</v>
       </c>
       <c r="B18" s="18" t="s">
         <v>1340</v>
@@ -76854,21 +77005,21 @@
         <v>2734</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>6624</v>
+        <v>6641</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H18" s="19" t="s">
-        <v>6625</v>
+        <v>6642</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>6626</v>
+        <v>6643</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>1340</v>
@@ -76877,48 +77028,48 @@
         <v>5175</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>6627</v>
+        <v>6644</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>6575</v>
+        <v>6592</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H19" s="19"/>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>6628</v>
+        <v>6645</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>6629</v>
+        <v>6646</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>6630</v>
+        <v>6647</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>6576</v>
+        <v>6593</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>6631</v>
+        <v>6648</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>6632</v>
+        <v>6649</v>
       </c>
       <c r="B21" s="18" t="s">
         <v>1340</v>
@@ -76927,24 +77078,24 @@
         <v>5175</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>6633</v>
+        <v>6650</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>6634</v>
+        <v>6651</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>6635</v>
+        <v>6652</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>6636</v>
+        <v>6653</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>6632</v>
+        <v>6649</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>1340</v>
@@ -76953,96 +77104,96 @@
         <v>2149</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>6637</v>
+        <v>6654</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>6638</v>
+        <v>6655</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H22" s="19" t="s">
-        <v>6639</v>
+        <v>6656</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>6632</v>
+        <v>6649</v>
       </c>
       <c r="B23" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>6600</v>
+        <v>6617</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>6640</v>
+        <v>6657</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>6641</v>
+        <v>6658</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H23" s="19"/>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>6642</v>
+        <v>6659</v>
       </c>
       <c r="B24" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>6643</v>
+        <v>6660</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>6644</v>
+        <v>6661</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>6645</v>
+        <v>6662</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>6646</v>
+        <v>6663</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H24" s="19"/>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>6647</v>
+        <v>6664</v>
       </c>
       <c r="B25" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>6648</v>
+        <v>6665</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>6649</v>
+        <v>6666</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>6650</v>
+        <v>6667</v>
       </c>
       <c r="B26" s="18" t="s">
         <v>1340</v>
@@ -77054,21 +77205,21 @@
         <v>5370</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>6651</v>
+        <v>6668</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>6652</v>
+        <v>6669</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>6653</v>
+        <v>6670</v>
       </c>
       <c r="B27" s="18" t="s">
         <v>1340</v>
@@ -77077,76 +77228,76 @@
         <v>5175</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>6654</v>
+        <v>6671</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>6655</v>
+        <v>6672</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="s">
-        <v>6653</v>
+        <v>6670</v>
       </c>
       <c r="B28" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>6648</v>
+        <v>6665</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>6656</v>
+        <v>6673</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>6657</v>
+        <v>6674</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>6658</v>
+        <v>6675</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>6659</v>
+        <v>6676</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>6653</v>
+        <v>6670</v>
       </c>
       <c r="B29" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>6660</v>
+        <v>6677</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>6661</v>
+        <v>6678</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>6602</v>
+        <v>6619</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>6662</v>
+        <v>6679</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>6663</v>
+        <v>6680</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>6664</v>
+        <v>6681</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>6665</v>
+        <v>6682</v>
       </c>
       <c r="B30" s="18" t="s">
         <v>1340</v>
@@ -77155,50 +77306,50 @@
         <v>5217</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>6666</v>
+        <v>6683</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>6667</v>
+        <v>6684</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>6668</v>
+        <v>6685</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>6669</v>
+        <v>6686</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>6670</v>
+        <v>6687</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="18" t="s">
-        <v>6665</v>
+        <v>6682</v>
       </c>
       <c r="B31" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>6648</v>
+        <v>6665</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>6671</v>
+        <v>6688</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>6672</v>
+        <v>6689</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>6673</v>
+        <v>6690</v>
       </c>
       <c r="G31" s="19" t="s">
         <v>5837</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>6674</v>
+        <v>6691</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="18" t="s">
-        <v>6665</v>
+        <v>6682</v>
       </c>
       <c r="B32" s="18" t="s">
         <v>1340</v>
@@ -77210,21 +77361,21 @@
         <v>3515</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>6675</v>
+        <v>6692</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="18" t="s">
-        <v>6676</v>
+        <v>6693</v>
       </c>
       <c r="B33" s="18" t="s">
         <v>1340</v>
@@ -77233,156 +77384,156 @@
         <v>5252</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>6677</v>
+        <v>6694</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>6678</v>
+        <v>6695</v>
       </c>
       <c r="F33" s="19" t="s">
         <v>5859</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>6679</v>
+        <v>6696</v>
       </c>
       <c r="H33" s="19" t="s">
-        <v>6680</v>
+        <v>6697</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>6676</v>
+        <v>6693</v>
       </c>
       <c r="B34" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>6681</v>
+        <v>6698</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>6682</v>
+        <v>6699</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>6683</v>
+        <v>6700</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>6684</v>
+        <v>6701</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>6685</v>
+        <v>6702</v>
       </c>
       <c r="B35" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>6686</v>
+        <v>6703</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>6687</v>
+        <v>6704</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>6688</v>
+        <v>6705</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H35" s="19" t="s">
-        <v>6689</v>
+        <v>6706</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>6685</v>
+        <v>6702</v>
       </c>
       <c r="B36" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>6648</v>
+        <v>6665</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>6690</v>
+        <v>6707</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>6691</v>
+        <v>6708</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>6692</v>
+        <v>6709</v>
       </c>
       <c r="B37" s="18" t="s">
         <v>1340</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>6693</v>
+        <v>6710</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>6694</v>
+        <v>6711</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>6567</v>
+        <v>6584</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>6568</v>
+        <v>6585</v>
       </c>
       <c r="H37" s="19"/>
     </row>
     <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>6692</v>
+        <v>6709</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>6695</v>
+        <v>6712</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>6545</v>
+        <v>6562</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>6696</v>
+        <v>6713</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>6697</v>
+        <v>6714</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>6577</v>
+        <v>6594</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>6698</v>
+        <v>6715</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>6699</v>
+        <v>6716</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>6700</v>
+        <v>6717</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>6701</v>
+        <v>6718</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>6702</v>
+        <v>6719</v>
       </c>
       <c r="D39" s="19" t="s">
         <v>5797</v>
@@ -77391,76 +77542,76 @@
         <v>161</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>6703</v>
+        <v>6720</v>
       </c>
       <c r="G39" s="19" t="s">
         <v>161</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>6704</v>
+        <v>6721</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>6700</v>
+        <v>6717</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>6701</v>
+        <v>6718</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>6702</v>
+        <v>6719</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>6705</v>
+        <v>6722</v>
       </c>
       <c r="E40" s="18" t="s">
         <v>161</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>6706</v>
+        <v>6723</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>6707</v>
+        <v>6724</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>6708</v>
+        <v>6725</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>6589</v>
+        <v>6606</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>6701</v>
+        <v>6718</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>6709</v>
+        <v>6726</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>6710</v>
+        <v>6727</v>
       </c>
       <c r="E41" s="18" t="s">
         <v>161</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>6711</v>
+        <v>6728</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>6712</v>
+        <v>6729</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>6713</v>
+        <v>6730</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="18" t="s">
-        <v>6595</v>
+        <v>6612</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>6701</v>
+        <v>6718</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>6714</v>
+        <v>6731</v>
       </c>
       <c r="D42" s="19" t="s">
         <v>4354</v>
@@ -77469,50 +77620,50 @@
         <v>161</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>6715</v>
+        <v>6732</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>6716</v>
+        <v>6733</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>6717</v>
+        <v>6734</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
+        <v>6735</v>
+      </c>
+      <c r="B43" s="18" t="s">
         <v>6718</v>
       </c>
-      <c r="B43" s="18" t="s">
-        <v>6701</v>
-      </c>
       <c r="C43" s="19" t="s">
-        <v>6719</v>
+        <v>6736</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>6720</v>
+        <v>6737</v>
       </c>
       <c r="E43" s="18" t="s">
         <v>161</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>6711</v>
+        <v>6728</v>
       </c>
       <c r="G43" s="19" t="s">
         <v>161</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>6721</v>
+        <v>6738</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
+        <v>6735</v>
+      </c>
+      <c r="B44" s="18" t="s">
         <v>6718</v>
       </c>
-      <c r="B44" s="18" t="s">
-        <v>6701</v>
-      </c>
       <c r="C44" s="19" t="s">
-        <v>6719</v>
+        <v>6736</v>
       </c>
       <c r="D44" s="19" t="s">
         <v>2782</v>
@@ -77521,148 +77672,148 @@
         <v>161</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>6711</v>
+        <v>6728</v>
       </c>
       <c r="G44" s="19" t="s">
         <v>161</v>
       </c>
       <c r="H44" s="19" t="s">
-        <v>6722</v>
+        <v>6739</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
-        <v>6608</v>
+        <v>6625</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>6723</v>
+        <v>6740</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>6724</v>
+        <v>6741</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>6725</v>
+        <v>6742</v>
       </c>
       <c r="E45" s="18" t="s">
         <v>161</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>6726</v>
+        <v>6743</v>
       </c>
       <c r="G45" s="19" t="s">
         <v>161</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>6727</v>
+        <v>6744</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>6728</v>
+        <v>6745</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>6723</v>
+        <v>6740</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>6729</v>
+        <v>6746</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>6730</v>
+        <v>6747</v>
       </c>
       <c r="E46" s="18" t="s">
         <v>1036</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>6731</v>
+        <v>6748</v>
       </c>
       <c r="G46" s="19" t="s">
         <v>161</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>6732</v>
+        <v>6749</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="s">
-        <v>6733</v>
+        <v>6750</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>6723</v>
+        <v>6740</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>6734</v>
+        <v>6751</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>6735</v>
+        <v>6752</v>
       </c>
       <c r="E47" s="18" t="s">
-        <v>6736</v>
+        <v>6753</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>6737</v>
+        <v>6754</v>
       </c>
       <c r="G47" s="19" t="s">
         <v>161</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>6738</v>
+        <v>6755</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="s">
-        <v>6628</v>
+        <v>6645</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>6723</v>
+        <v>6740</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>6739</v>
+        <v>6756</v>
       </c>
       <c r="D48" s="19" t="s">
-        <v>6740</v>
+        <v>6757</v>
       </c>
       <c r="E48" s="18" t="s">
-        <v>6741</v>
+        <v>6758</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>6742</v>
+        <v>6759</v>
       </c>
       <c r="G48" s="19" t="s">
         <v>5862</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>6743</v>
+        <v>6760</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="s">
-        <v>6632</v>
+        <v>6649</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>6723</v>
+        <v>6740</v>
       </c>
       <c r="C49" s="19" t="s">
-        <v>6744</v>
+        <v>6761</v>
       </c>
       <c r="D49" s="19" t="s">
         <v>2682</v>
       </c>
       <c r="E49" s="18" t="s">
-        <v>6745</v>
+        <v>6762</v>
       </c>
       <c r="F49" s="19" t="s">
-        <v>6746</v>
+        <v>6763</v>
       </c>
       <c r="G49" s="19" t="s">
-        <v>6747</v>
+        <v>6764</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>6748</v>
+        <v>6765</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="29" t="s">
-        <v>6749</v>
+        <v>6766</v>
       </c>
       <c r="B51" s="29"/>
       <c r="C51" s="29"/>
@@ -77710,41 +77861,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
-        <v>6750</v>
+        <v>6767</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
-        <v>6751</v>
+        <v>6768</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>6752</v>
+        <v>6769</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="35" t="s">
-        <v>6753</v>
+        <v>6770</v>
       </c>
       <c r="B5" s="35" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>6754</v>
+        <v>6771</v>
       </c>
       <c r="D5" s="35" t="s">
-        <v>6755</v>
+        <v>6772</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>6756</v>
+        <v>6773</v>
       </c>
       <c r="F5" s="35" t="s">
         <v>5820</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>6757</v>
+        <v>6774</v>
       </c>
       <c r="H5" s="35" t="s">
         <v>13</v>
@@ -77752,161 +77903,161 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="s">
-        <v>6758</v>
+        <v>6775</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>6759</v>
+        <v>6776</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>6238</v>
+        <v>6239</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>6760</v>
+        <v>6777</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>6761</v>
+        <v>6778</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G6" s="38"/>
       <c r="H6" s="38"/>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="36" t="s">
-        <v>6763</v>
+        <v>6780</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>6759</v>
+        <v>6776</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>6764</v>
+        <v>6781</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>6765</v>
+        <v>6782</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>6766</v>
+        <v>6783</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G7" s="38"/>
       <c r="H7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="36" t="s">
-        <v>6767</v>
+        <v>6784</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>6759</v>
+        <v>6776</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>6768</v>
+        <v>6785</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>6769</v>
+        <v>6786</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>6770</v>
+        <v>6787</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G8" s="38"/>
       <c r="H8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="36" t="s">
-        <v>6771</v>
+        <v>6788</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>6759</v>
+        <v>6776</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>6772</v>
+        <v>6789</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>6773</v>
+        <v>6790</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>6774</v>
+        <v>6791</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G9" s="38"/>
       <c r="H9" s="38"/>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="36" t="s">
-        <v>6775</v>
+        <v>6792</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>6776</v>
+        <v>6793</v>
       </c>
       <c r="C10" s="37" t="s">
         <v>5884</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>6777</v>
+        <v>6794</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>6778</v>
+        <v>6795</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G10" s="38"/>
       <c r="H10" s="38"/>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="36" t="s">
-        <v>6779</v>
+        <v>6796</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>6776</v>
+        <v>6793</v>
       </c>
       <c r="C11" s="37" t="s">
         <v>59</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>6781</v>
+        <v>6798</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G11" s="38"/>
       <c r="H11" s="38"/>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>6782</v>
+        <v>6799</v>
       </c>
       <c r="B12" s="37" t="s">
         <v>6034</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>6224</v>
+        <v>6225</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>6783</v>
+        <v>6800</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G12" s="38"/>
       <c r="H12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="36" t="s">
-        <v>6784</v>
+        <v>6801</v>
       </c>
       <c r="B13" s="37" t="s">
         <v>6034</v>
@@ -77915,42 +78066,42 @@
         <v>123</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>6785</v>
+        <v>6802</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>6786</v>
+        <v>6803</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G13" s="38"/>
       <c r="H13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="s">
-        <v>6788</v>
+        <v>6805</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>6789</v>
+        <v>6806</v>
       </c>
       <c r="C14" s="37" t="s">
         <v>107</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>6790</v>
+        <v>6807</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G14" s="38"/>
       <c r="H14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="s">
-        <v>6791</v>
+        <v>6808</v>
       </c>
       <c r="B15" s="37" t="s">
         <v>6034</v>
@@ -77959,20 +78110,20 @@
         <v>130</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>6792</v>
+        <v>6809</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>6793</v>
+        <v>6810</v>
       </c>
       <c r="F15" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G15" s="38"/>
       <c r="H15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="s">
-        <v>6794</v>
+        <v>6811</v>
       </c>
       <c r="B16" s="37" t="s">
         <v>6034</v>
@@ -77981,42 +78132,42 @@
         <v>287</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>6795</v>
+        <v>6812</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>6796</v>
+        <v>6813</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>6797</v>
+        <v>6814</v>
       </c>
       <c r="G16" s="38"/>
       <c r="H16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="36" t="s">
-        <v>6798</v>
+        <v>6815</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>6789</v>
+        <v>6806</v>
       </c>
       <c r="C17" s="37" t="s">
         <v>100</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>6799</v>
+        <v>6816</v>
       </c>
       <c r="F17" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G17" s="38"/>
       <c r="H17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="36" t="s">
-        <v>6800</v>
+        <v>6817</v>
       </c>
       <c r="B18" s="37" t="s">
         <v>6034</v>
@@ -78025,79 +78176,79 @@
         <v>5023</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>6801</v>
+        <v>6818</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>6797</v>
+        <v>6814</v>
       </c>
       <c r="G18" s="38"/>
       <c r="H18" s="38"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="36" t="s">
-        <v>6802</v>
+        <v>6819</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>6803</v>
+        <v>6820</v>
       </c>
       <c r="C19" s="37" t="s">
+        <v>6821</v>
+      </c>
+      <c r="D19" s="37" t="s">
+        <v>6797</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>6822</v>
+      </c>
+      <c r="F19" s="37" t="s">
         <v>6804</v>
-      </c>
-      <c r="D19" s="37" t="s">
-        <v>6780</v>
-      </c>
-      <c r="E19" s="37" t="s">
-        <v>6805</v>
-      </c>
-      <c r="F19" s="37" t="s">
-        <v>6787</v>
       </c>
       <c r="G19" s="38"/>
       <c r="H19" s="38"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="36" t="s">
-        <v>6806</v>
+        <v>6823</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>6803</v>
+        <v>6820</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>6807</v>
+        <v>6824</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>6808</v>
+        <v>6825</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G20" s="38"/>
       <c r="H20" s="38"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="36" t="s">
-        <v>6809</v>
+        <v>6826</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>6803</v>
+        <v>6820</v>
       </c>
       <c r="C21" s="37" t="s">
         <v>59</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>6810</v>
+        <v>6827</v>
       </c>
       <c r="F21" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G21" s="38"/>
       <c r="H21" s="38"/>
@@ -78107,48 +78258,48 @@
         <v>6042</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>6803</v>
+        <v>6820</v>
       </c>
       <c r="C22" s="37" t="s">
-        <v>6811</v>
+        <v>6828</v>
       </c>
       <c r="D22" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>6812</v>
+        <v>6829</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G22" s="38"/>
       <c r="H22" s="38"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="36" t="s">
-        <v>6813</v>
+        <v>6830</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>6803</v>
+        <v>6820</v>
       </c>
       <c r="C23" s="37" t="s">
+        <v>6831</v>
+      </c>
+      <c r="D23" s="37" t="s">
+        <v>6832</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>6833</v>
+      </c>
+      <c r="F23" s="37" t="s">
         <v>6814</v>
-      </c>
-      <c r="D23" s="37" t="s">
-        <v>6815</v>
-      </c>
-      <c r="E23" s="37" t="s">
-        <v>6816</v>
-      </c>
-      <c r="F23" s="37" t="s">
-        <v>6797</v>
       </c>
       <c r="G23" s="38"/>
       <c r="H23" s="38"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="36" t="s">
-        <v>6817</v>
+        <v>6834</v>
       </c>
       <c r="B24" s="37" t="s">
         <v>6034</v>
@@ -78157,152 +78308,152 @@
         <v>42</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>6818</v>
+        <v>6835</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G24" s="38"/>
       <c r="H24" s="38"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="36" t="s">
-        <v>6819</v>
+        <v>6836</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>6803</v>
+        <v>6820</v>
       </c>
       <c r="C25" s="37" t="s">
         <v>255</v>
       </c>
       <c r="D25" s="37" t="s">
-        <v>6815</v>
+        <v>6832</v>
       </c>
       <c r="E25" s="37" t="s">
-        <v>6820</v>
+        <v>6837</v>
       </c>
       <c r="F25" s="37" t="s">
-        <v>6797</v>
+        <v>6814</v>
       </c>
       <c r="G25" s="38"/>
       <c r="H25" s="38"/>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="36" t="s">
-        <v>6821</v>
+        <v>6838</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>6822</v>
+        <v>6839</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>6823</v>
+        <v>6840</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>6824</v>
+        <v>6841</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>6825</v>
+        <v>6842</v>
       </c>
       <c r="F26" s="37" t="s">
-        <v>6762</v>
+        <v>6779</v>
       </c>
       <c r="G26" s="38"/>
       <c r="H26" s="38"/>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="36" t="s">
-        <v>6826</v>
+        <v>6843</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>6822</v>
+        <v>6839</v>
       </c>
       <c r="C27" s="37" t="s">
-        <v>6827</v>
+        <v>6844</v>
       </c>
       <c r="D27" s="37" t="s">
-        <v>6828</v>
+        <v>6845</v>
       </c>
       <c r="E27" s="37" t="s">
-        <v>6829</v>
+        <v>6846</v>
       </c>
       <c r="F27" s="37" t="s">
-        <v>6797</v>
+        <v>6814</v>
       </c>
       <c r="G27" s="38"/>
       <c r="H27" s="38"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="36" t="s">
-        <v>6830</v>
+        <v>6847</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>6822</v>
+        <v>6839</v>
       </c>
       <c r="C28" s="37" t="s">
         <v>745</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>6828</v>
+        <v>6845</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>6831</v>
+        <v>6848</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>6797</v>
+        <v>6814</v>
       </c>
       <c r="G28" s="38"/>
       <c r="H28" s="38"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="36" t="s">
-        <v>6832</v>
+        <v>6849</v>
       </c>
       <c r="B29" s="37" t="s">
-        <v>6833</v>
+        <v>6850</v>
       </c>
       <c r="C29" s="37" t="s">
         <v>25</v>
       </c>
       <c r="D29" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E29" s="37" t="s">
-        <v>6834</v>
+        <v>6851</v>
       </c>
       <c r="F29" s="37" t="s">
-        <v>6787</v>
+        <v>6804</v>
       </c>
       <c r="G29" s="38"/>
       <c r="H29" s="38"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="36" t="s">
-        <v>6835</v>
+        <v>6852</v>
       </c>
       <c r="B30" s="37" t="s">
-        <v>6833</v>
+        <v>6850</v>
       </c>
       <c r="C30" s="37" t="s">
-        <v>6836</v>
+        <v>6853</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>6780</v>
+        <v>6797</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>6837</v>
+        <v>6854</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>6797</v>
+        <v>6814</v>
       </c>
       <c r="G30" s="38"/>
       <c r="H30" s="38"/>
     </row>
     <row r="32" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="40" t="s">
-        <v>6838</v>
+        <v>6855</v>
       </c>
     </row>
   </sheetData>

</xml_diff>